<commit_message>
Organizar mejor las rutas
</commit_message>
<xml_diff>
--- a/Planificacion_Proyecto_Nautico_Poseidon.xlsx
+++ b/Planificacion_Proyecto_Nautico_Poseidon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\UNI\2026-2\Desarrollo\PF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0880032B-FDF3-4B7F-95DA-1F0504E13B98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45E92AE2-55E5-470F-A8C5-BCD9CA11A092}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1086,6 +1086,24 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -1094,18 +1112,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1120,12 +1126,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1450,32 +1450,32 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="31" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
+      <c r="C1" s="31"/>
+      <c r="D1" s="31"/>
     </row>
     <row r="2" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
+      <c r="C2" s="31"/>
+      <c r="D2" s="31"/>
     </row>
     <row r="3" spans="1:9" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="36" t="str">
+      <c r="B3" s="31" t="str">
         <f>EQUIPO!$B$7</f>
         <v>Jose Espinoza Rivadeneira</v>
       </c>
-      <c r="C3" s="36"/>
-      <c r="D3" s="36"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
     </row>
     <row r="4" spans="1:9" ht="9.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:9" ht="33.75" customHeight="1" x14ac:dyDescent="0.3">
@@ -1508,13 +1508,13 @@
       </c>
     </row>
     <row r="6" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="33" t="s">
+      <c r="A6" s="32" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="3">
         <v>1</v>
       </c>
-      <c r="C6" s="43" t="s">
+      <c r="C6" s="33" t="s">
         <v>15</v>
       </c>
       <c r="D6" s="4" t="s">
@@ -1538,7 +1538,7 @@
       </c>
     </row>
     <row r="7" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="33"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="5">
         <v>1</v>
       </c>
@@ -1555,7 +1555,7 @@
       <c r="I7" s="34"/>
     </row>
     <row r="8" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="33"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="5">
         <v>1</v>
       </c>
@@ -1572,7 +1572,7 @@
       <c r="I8" s="34"/>
     </row>
     <row r="9" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="33"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="5">
         <v>1</v>
       </c>
@@ -1581,7 +1581,7 @@
         <v>23</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F9" s="34"/>
       <c r="G9" s="35"/>
@@ -1589,11 +1589,11 @@
       <c r="I9" s="34"/>
     </row>
     <row r="10" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="33"/>
+      <c r="A10" s="32"/>
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="43" t="s">
+      <c r="C10" s="33" t="s">
         <v>24</v>
       </c>
       <c r="D10" s="4" t="s">
@@ -1617,7 +1617,7 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="33"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5">
         <v>1</v>
       </c>
@@ -1634,7 +1634,7 @@
       <c r="I11" s="34"/>
     </row>
     <row r="12" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="33"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="5">
         <v>1</v>
       </c>
@@ -1651,7 +1651,7 @@
       <c r="I12" s="34"/>
     </row>
     <row r="13" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="33"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="5">
         <v>1</v>
       </c>
@@ -1668,11 +1668,11 @@
       <c r="I13" s="34"/>
     </row>
     <row r="14" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="3">
         <v>1</v>
       </c>
-      <c r="C14" s="43" t="s">
+      <c r="C14" s="33" t="s">
         <v>31</v>
       </c>
       <c r="D14" s="4" t="s">
@@ -1696,7 +1696,7 @@
       </c>
     </row>
     <row r="15" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="33"/>
+      <c r="A15" s="32"/>
       <c r="B15" s="5">
         <v>1</v>
       </c>
@@ -1713,7 +1713,7 @@
       <c r="I15" s="34"/>
     </row>
     <row r="16" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="33"/>
+      <c r="A16" s="32"/>
       <c r="B16" s="5">
         <v>1</v>
       </c>
@@ -1730,7 +1730,7 @@
       <c r="I16" s="34"/>
     </row>
     <row r="17" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="33"/>
+      <c r="A17" s="32"/>
       <c r="B17" s="5">
         <v>1</v>
       </c>
@@ -1739,7 +1739,7 @@
         <v>37</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F17" s="34"/>
       <c r="G17" s="35"/>
@@ -1747,11 +1747,11 @@
       <c r="I17" s="34"/>
     </row>
     <row r="18" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="33"/>
+      <c r="A18" s="32"/>
       <c r="B18" s="3">
         <v>1</v>
       </c>
-      <c r="C18" s="43" t="s">
+      <c r="C18" s="33" t="s">
         <v>38</v>
       </c>
       <c r="D18" s="4" t="s">
@@ -1775,7 +1775,7 @@
       </c>
     </row>
     <row r="19" spans="1:9" ht="67.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="33"/>
+      <c r="A19" s="32"/>
       <c r="B19" s="5">
         <v>1</v>
       </c>
@@ -1784,7 +1784,7 @@
         <v>41</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="F19" s="34"/>
       <c r="G19" s="35"/>
@@ -1792,7 +1792,7 @@
       <c r="I19" s="34"/>
     </row>
     <row r="20" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="33"/>
+      <c r="A20" s="32"/>
       <c r="B20" s="5">
         <v>1</v>
       </c>
@@ -1809,7 +1809,7 @@
       <c r="I20" s="34"/>
     </row>
     <row r="21" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="33"/>
+      <c r="A21" s="32"/>
       <c r="B21" s="5">
         <v>1</v>
       </c>
@@ -1826,11 +1826,11 @@
       <c r="I21" s="34"/>
     </row>
     <row r="22" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="33"/>
+      <c r="A22" s="32"/>
       <c r="B22" s="3">
         <v>1</v>
       </c>
-      <c r="C22" s="43" t="s">
+      <c r="C22" s="33" t="s">
         <v>44</v>
       </c>
       <c r="D22" s="4" t="s">
@@ -1854,7 +1854,7 @@
       </c>
     </row>
     <row r="23" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="33"/>
+      <c r="A23" s="32"/>
       <c r="B23" s="5">
         <v>1</v>
       </c>
@@ -1871,7 +1871,7 @@
       <c r="I23" s="34"/>
     </row>
     <row r="24" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="33"/>
+      <c r="A24" s="32"/>
       <c r="B24" s="5">
         <v>1</v>
       </c>
@@ -1888,7 +1888,7 @@
       <c r="I24" s="34"/>
     </row>
     <row r="25" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="33"/>
+      <c r="A25" s="32"/>
       <c r="B25" s="5">
         <v>1</v>
       </c>
@@ -1896,7 +1896,7 @@
       <c r="D25" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="E25" s="42" t="s">
+      <c r="E25" s="30" t="s">
         <v>230</v>
       </c>
       <c r="F25" s="34"/>
@@ -1905,13 +1905,13 @@
       <c r="I25" s="34"/>
     </row>
     <row r="26" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="30" t="s">
+      <c r="A26" s="36" t="s">
         <v>50</v>
       </c>
       <c r="B26" s="7">
         <v>2</v>
       </c>
-      <c r="C26" s="31" t="s">
+      <c r="C26" s="37" t="s">
         <v>51</v>
       </c>
       <c r="D26" s="8" t="s">
@@ -1920,77 +1920,77 @@
       <c r="E26" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="31" t="s">
+      <c r="F26" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="G26" s="32" t="s">
+      <c r="G26" s="38" t="s">
         <v>54</v>
       </c>
-      <c r="H26" s="32" t="str">
+      <c r="H26" s="38" t="str">
         <f>EQUIPO!$B$7</f>
         <v>Jose Espinoza Rivadeneira</v>
       </c>
-      <c r="I26" s="31" t="s">
+      <c r="I26" s="37" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="30"/>
+      <c r="A27" s="36"/>
       <c r="B27" s="9">
         <v>2</v>
       </c>
-      <c r="C27" s="31"/>
+      <c r="C27" s="37"/>
       <c r="D27" s="10" t="s">
         <v>55</v>
       </c>
       <c r="E27" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F27" s="31"/>
-      <c r="G27" s="32"/>
-      <c r="H27" s="32"/>
-      <c r="I27" s="31"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="37"/>
     </row>
     <row r="28" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="30"/>
+      <c r="A28" s="36"/>
       <c r="B28" s="9">
         <v>2</v>
       </c>
-      <c r="C28" s="31"/>
+      <c r="C28" s="37"/>
       <c r="D28" s="10" t="s">
         <v>56</v>
       </c>
       <c r="E28" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F28" s="31"/>
-      <c r="G28" s="32"/>
-      <c r="H28" s="32"/>
-      <c r="I28" s="31"/>
+      <c r="F28" s="37"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="37"/>
     </row>
     <row r="29" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="30"/>
+      <c r="A29" s="36"/>
       <c r="B29" s="9">
         <v>2</v>
       </c>
-      <c r="C29" s="31"/>
+      <c r="C29" s="37"/>
       <c r="D29" s="10" t="s">
         <v>57</v>
       </c>
       <c r="E29" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F29" s="31"/>
-      <c r="G29" s="32"/>
-      <c r="H29" s="32"/>
-      <c r="I29" s="31"/>
+      <c r="F29" s="37"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="37"/>
     </row>
     <row r="30" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="30"/>
+      <c r="A30" s="36"/>
       <c r="B30" s="7">
         <v>2</v>
       </c>
-      <c r="C30" s="31" t="s">
+      <c r="C30" s="37" t="s">
         <v>58</v>
       </c>
       <c r="D30" s="8" t="s">
@@ -1999,73 +1999,73 @@
       <c r="E30" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F30" s="31" t="s">
+      <c r="F30" s="37" t="s">
         <v>53</v>
       </c>
-      <c r="G30" s="32" t="s">
+      <c r="G30" s="38" t="s">
         <v>60</v>
       </c>
-      <c r="H30" s="32" t="str">
+      <c r="H30" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I30" s="31" t="s">
+      <c r="I30" s="37" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="30"/>
+      <c r="A31" s="36"/>
       <c r="B31" s="9">
         <v>2</v>
       </c>
-      <c r="C31" s="31"/>
+      <c r="C31" s="37"/>
       <c r="D31" s="10" t="s">
         <v>61</v>
       </c>
       <c r="E31" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F31" s="31"/>
-      <c r="G31" s="32"/>
-      <c r="H31" s="32"/>
-      <c r="I31" s="31"/>
+      <c r="F31" s="37"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="37"/>
     </row>
     <row r="32" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="30"/>
+      <c r="A32" s="36"/>
       <c r="B32" s="9">
         <v>2</v>
       </c>
-      <c r="C32" s="31"/>
+      <c r="C32" s="37"/>
       <c r="D32" s="10" t="s">
         <v>62</v>
       </c>
       <c r="E32" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F32" s="31"/>
-      <c r="G32" s="32"/>
-      <c r="H32" s="32"/>
-      <c r="I32" s="31"/>
+      <c r="F32" s="37"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="37"/>
     </row>
     <row r="33" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="30"/>
+      <c r="A33" s="36"/>
       <c r="B33" s="9">
         <v>2</v>
       </c>
-      <c r="C33" s="31"/>
+      <c r="C33" s="37"/>
       <c r="D33" s="10" t="s">
         <v>63</v>
       </c>
       <c r="E33" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F33" s="31"/>
-      <c r="G33" s="32"/>
-      <c r="H33" s="32"/>
-      <c r="I33" s="31"/>
+      <c r="F33" s="37"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="37"/>
     </row>
     <row r="34" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="33" t="s">
+      <c r="A34" s="32" t="s">
         <v>64</v>
       </c>
       <c r="B34" s="3">
@@ -2095,7 +2095,7 @@
       </c>
     </row>
     <row r="35" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="33"/>
+      <c r="A35" s="32"/>
       <c r="B35" s="5">
         <v>3</v>
       </c>
@@ -2112,7 +2112,7 @@
       <c r="I35" s="34"/>
     </row>
     <row r="36" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="33"/>
+      <c r="A36" s="32"/>
       <c r="B36" s="5">
         <v>3</v>
       </c>
@@ -2129,7 +2129,7 @@
       <c r="I36" s="34"/>
     </row>
     <row r="37" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="33"/>
+      <c r="A37" s="32"/>
       <c r="B37" s="5">
         <v>3</v>
       </c>
@@ -2146,7 +2146,7 @@
       <c r="I37" s="34"/>
     </row>
     <row r="38" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="33"/>
+      <c r="A38" s="32"/>
       <c r="B38" s="3">
         <v>3</v>
       </c>
@@ -2174,7 +2174,7 @@
       </c>
     </row>
     <row r="39" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="33"/>
+      <c r="A39" s="32"/>
       <c r="B39" s="5">
         <v>3</v>
       </c>
@@ -2191,7 +2191,7 @@
       <c r="I39" s="34"/>
     </row>
     <row r="40" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="33"/>
+      <c r="A40" s="32"/>
       <c r="B40" s="5">
         <v>3</v>
       </c>
@@ -2208,7 +2208,7 @@
       <c r="I40" s="34"/>
     </row>
     <row r="41" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="33"/>
+      <c r="A41" s="32"/>
       <c r="B41" s="5">
         <v>3</v>
       </c>
@@ -2225,7 +2225,7 @@
       <c r="I41" s="34"/>
     </row>
     <row r="42" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="33"/>
+      <c r="A42" s="32"/>
       <c r="B42" s="5">
         <v>3</v>
       </c>
@@ -2242,7 +2242,7 @@
       <c r="I42" s="34"/>
     </row>
     <row r="43" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="33"/>
+      <c r="A43" s="32"/>
       <c r="B43" s="3">
         <v>3</v>
       </c>
@@ -2270,7 +2270,7 @@
       </c>
     </row>
     <row r="44" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="33"/>
+      <c r="A44" s="32"/>
       <c r="B44" s="5">
         <v>3</v>
       </c>
@@ -2287,7 +2287,7 @@
       <c r="I44" s="34"/>
     </row>
     <row r="45" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="33"/>
+      <c r="A45" s="32"/>
       <c r="B45" s="5">
         <v>3</v>
       </c>
@@ -2304,7 +2304,7 @@
       <c r="I45" s="34"/>
     </row>
     <row r="46" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="33"/>
+      <c r="A46" s="32"/>
       <c r="B46" s="5">
         <v>3</v>
       </c>
@@ -2321,13 +2321,13 @@
       <c r="I46" s="34"/>
     </row>
     <row r="47" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="36" t="s">
         <v>86</v>
       </c>
       <c r="B47" s="7">
         <v>4</v>
       </c>
-      <c r="C47" s="31" t="s">
+      <c r="C47" s="37" t="s">
         <v>87</v>
       </c>
       <c r="D47" s="8" t="s">
@@ -2336,77 +2336,77 @@
       <c r="E47" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F47" s="31" t="s">
+      <c r="F47" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G47" s="32" t="s">
+      <c r="G47" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="H47" s="32" t="str">
+      <c r="H47" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I47" s="31" t="s">
+      <c r="I47" s="37" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="48" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="30"/>
+      <c r="A48" s="36"/>
       <c r="B48" s="9">
         <v>4</v>
       </c>
-      <c r="C48" s="31"/>
+      <c r="C48" s="37"/>
       <c r="D48" s="10" t="s">
         <v>90</v>
       </c>
       <c r="E48" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F48" s="31"/>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="31"/>
+      <c r="F48" s="37"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="37"/>
     </row>
     <row r="49" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="30"/>
+      <c r="A49" s="36"/>
       <c r="B49" s="9">
         <v>4</v>
       </c>
-      <c r="C49" s="31"/>
+      <c r="C49" s="37"/>
       <c r="D49" s="10" t="s">
         <v>91</v>
       </c>
       <c r="E49" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F49" s="31"/>
-      <c r="G49" s="32"/>
-      <c r="H49" s="32"/>
-      <c r="I49" s="31"/>
+      <c r="F49" s="37"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="37"/>
     </row>
     <row r="50" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="30"/>
+      <c r="A50" s="36"/>
       <c r="B50" s="9">
         <v>4</v>
       </c>
-      <c r="C50" s="31"/>
+      <c r="C50" s="37"/>
       <c r="D50" s="10" t="s">
         <v>92</v>
       </c>
       <c r="E50" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F50" s="31"/>
-      <c r="G50" s="32"/>
-      <c r="H50" s="32"/>
-      <c r="I50" s="31"/>
+      <c r="F50" s="37"/>
+      <c r="G50" s="38"/>
+      <c r="H50" s="38"/>
+      <c r="I50" s="37"/>
     </row>
     <row r="51" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="30"/>
+      <c r="A51" s="36"/>
       <c r="B51" s="7">
         <v>4</v>
       </c>
-      <c r="C51" s="31" t="s">
+      <c r="C51" s="37" t="s">
         <v>93</v>
       </c>
       <c r="D51" s="8" t="s">
@@ -2415,77 +2415,77 @@
       <c r="E51" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F51" s="31" t="s">
+      <c r="F51" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G51" s="32" t="s">
+      <c r="G51" s="38" t="s">
         <v>95</v>
       </c>
-      <c r="H51" s="32" t="str">
+      <c r="H51" s="38" t="str">
         <f>EQUIPO!$B$7</f>
         <v>Jose Espinoza Rivadeneira</v>
       </c>
-      <c r="I51" s="31" t="s">
+      <c r="I51" s="37" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="30"/>
+      <c r="A52" s="36"/>
       <c r="B52" s="9">
         <v>4</v>
       </c>
-      <c r="C52" s="31"/>
+      <c r="C52" s="37"/>
       <c r="D52" s="10" t="s">
         <v>96</v>
       </c>
       <c r="E52" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F52" s="31"/>
-      <c r="G52" s="32"/>
-      <c r="H52" s="32"/>
-      <c r="I52" s="31"/>
+      <c r="F52" s="37"/>
+      <c r="G52" s="38"/>
+      <c r="H52" s="38"/>
+      <c r="I52" s="37"/>
     </row>
     <row r="53" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="30"/>
+      <c r="A53" s="36"/>
       <c r="B53" s="9">
         <v>4</v>
       </c>
-      <c r="C53" s="31"/>
+      <c r="C53" s="37"/>
       <c r="D53" s="10" t="s">
         <v>97</v>
       </c>
       <c r="E53" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F53" s="31"/>
-      <c r="G53" s="32"/>
-      <c r="H53" s="32"/>
-      <c r="I53" s="31"/>
+      <c r="F53" s="37"/>
+      <c r="G53" s="38"/>
+      <c r="H53" s="38"/>
+      <c r="I53" s="37"/>
     </row>
     <row r="54" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="30"/>
+      <c r="A54" s="36"/>
       <c r="B54" s="9">
         <v>4</v>
       </c>
-      <c r="C54" s="31"/>
+      <c r="C54" s="37"/>
       <c r="D54" s="10" t="s">
         <v>98</v>
       </c>
       <c r="E54" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F54" s="31"/>
-      <c r="G54" s="32"/>
-      <c r="H54" s="32"/>
-      <c r="I54" s="31"/>
+      <c r="F54" s="37"/>
+      <c r="G54" s="38"/>
+      <c r="H54" s="38"/>
+      <c r="I54" s="37"/>
     </row>
     <row r="55" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="30"/>
+      <c r="A55" s="36"/>
       <c r="B55" s="7">
         <v>4</v>
       </c>
-      <c r="C55" s="31" t="s">
+      <c r="C55" s="37" t="s">
         <v>99</v>
       </c>
       <c r="D55" s="8" t="s">
@@ -2494,73 +2494,73 @@
       <c r="E55" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F55" s="31" t="s">
+      <c r="F55" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G55" s="32" t="s">
+      <c r="G55" s="38" t="s">
         <v>101</v>
       </c>
-      <c r="H55" s="32" t="str">
+      <c r="H55" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I55" s="31" t="s">
+      <c r="I55" s="37" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="56" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="30"/>
+      <c r="A56" s="36"/>
       <c r="B56" s="9">
         <v>4</v>
       </c>
-      <c r="C56" s="31"/>
+      <c r="C56" s="37"/>
       <c r="D56" s="10" t="s">
         <v>102</v>
       </c>
       <c r="E56" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F56" s="31"/>
-      <c r="G56" s="32"/>
-      <c r="H56" s="32"/>
-      <c r="I56" s="31"/>
+      <c r="F56" s="37"/>
+      <c r="G56" s="38"/>
+      <c r="H56" s="38"/>
+      <c r="I56" s="37"/>
     </row>
     <row r="57" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="30"/>
+      <c r="A57" s="36"/>
       <c r="B57" s="9">
         <v>4</v>
       </c>
-      <c r="C57" s="31"/>
+      <c r="C57" s="37"/>
       <c r="D57" s="10" t="s">
         <v>103</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F57" s="31"/>
-      <c r="G57" s="32"/>
-      <c r="H57" s="32"/>
-      <c r="I57" s="31"/>
+      <c r="F57" s="37"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="37"/>
     </row>
     <row r="58" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="30"/>
+      <c r="A58" s="36"/>
       <c r="B58" s="9">
         <v>4</v>
       </c>
-      <c r="C58" s="31"/>
+      <c r="C58" s="37"/>
       <c r="D58" s="10" t="s">
         <v>104</v>
       </c>
       <c r="E58" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F58" s="31"/>
-      <c r="G58" s="32"/>
-      <c r="H58" s="32"/>
-      <c r="I58" s="31"/>
+      <c r="F58" s="37"/>
+      <c r="G58" s="38"/>
+      <c r="H58" s="38"/>
+      <c r="I58" s="37"/>
     </row>
     <row r="59" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="33" t="s">
+      <c r="A59" s="32" t="s">
         <v>105</v>
       </c>
       <c r="B59" s="3">
@@ -2590,7 +2590,7 @@
       </c>
     </row>
     <row r="60" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="33"/>
+      <c r="A60" s="32"/>
       <c r="B60" s="5">
         <v>5</v>
       </c>
@@ -2607,7 +2607,7 @@
       <c r="I60" s="34"/>
     </row>
     <row r="61" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="33"/>
+      <c r="A61" s="32"/>
       <c r="B61" s="5">
         <v>5</v>
       </c>
@@ -2624,7 +2624,7 @@
       <c r="I61" s="34"/>
     </row>
     <row r="62" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="33"/>
+      <c r="A62" s="32"/>
       <c r="B62" s="5">
         <v>5</v>
       </c>
@@ -2641,7 +2641,7 @@
       <c r="I62" s="34"/>
     </row>
     <row r="63" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="33"/>
+      <c r="A63" s="32"/>
       <c r="B63" s="3">
         <v>5</v>
       </c>
@@ -2669,7 +2669,7 @@
       </c>
     </row>
     <row r="64" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="33"/>
+      <c r="A64" s="32"/>
       <c r="B64" s="5">
         <v>5</v>
       </c>
@@ -2686,7 +2686,7 @@
       <c r="I64" s="34"/>
     </row>
     <row r="65" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="33"/>
+      <c r="A65" s="32"/>
       <c r="B65" s="5">
         <v>5</v>
       </c>
@@ -2703,7 +2703,7 @@
       <c r="I65" s="34"/>
     </row>
     <row r="66" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="33"/>
+      <c r="A66" s="32"/>
       <c r="B66" s="5">
         <v>5</v>
       </c>
@@ -2720,7 +2720,7 @@
       <c r="I66" s="34"/>
     </row>
     <row r="67" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="33"/>
+      <c r="A67" s="32"/>
       <c r="B67" s="3">
         <v>5</v>
       </c>
@@ -2748,7 +2748,7 @@
       </c>
     </row>
     <row r="68" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="33"/>
+      <c r="A68" s="32"/>
       <c r="B68" s="5">
         <v>5</v>
       </c>
@@ -2765,7 +2765,7 @@
       <c r="I68" s="34"/>
     </row>
     <row r="69" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="33"/>
+      <c r="A69" s="32"/>
       <c r="B69" s="5">
         <v>5</v>
       </c>
@@ -2782,7 +2782,7 @@
       <c r="I69" s="34"/>
     </row>
     <row r="70" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="33"/>
+      <c r="A70" s="32"/>
       <c r="B70" s="5">
         <v>5</v>
       </c>
@@ -2799,13 +2799,13 @@
       <c r="I70" s="34"/>
     </row>
     <row r="71" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="30" t="s">
+      <c r="A71" s="36" t="s">
         <v>124</v>
       </c>
       <c r="B71" s="7">
         <v>6</v>
       </c>
-      <c r="C71" s="31" t="s">
+      <c r="C71" s="37" t="s">
         <v>125</v>
       </c>
       <c r="D71" s="8" t="s">
@@ -2814,77 +2814,77 @@
       <c r="E71" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F71" s="31" t="s">
+      <c r="F71" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G71" s="32" t="s">
+      <c r="G71" s="38" t="s">
         <v>127</v>
       </c>
-      <c r="H71" s="32" t="str">
+      <c r="H71" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I71" s="31" t="s">
+      <c r="I71" s="37" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="72" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="30"/>
+      <c r="A72" s="36"/>
       <c r="B72" s="9">
         <v>6</v>
       </c>
-      <c r="C72" s="31"/>
+      <c r="C72" s="37"/>
       <c r="D72" s="10" t="s">
         <v>129</v>
       </c>
       <c r="E72" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F72" s="31"/>
-      <c r="G72" s="32"/>
-      <c r="H72" s="32"/>
-      <c r="I72" s="31"/>
+      <c r="F72" s="37"/>
+      <c r="G72" s="38"/>
+      <c r="H72" s="38"/>
+      <c r="I72" s="37"/>
     </row>
     <row r="73" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="30"/>
+      <c r="A73" s="36"/>
       <c r="B73" s="9">
         <v>6</v>
       </c>
-      <c r="C73" s="31"/>
+      <c r="C73" s="37"/>
       <c r="D73" s="10" t="s">
         <v>130</v>
       </c>
       <c r="E73" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F73" s="31"/>
-      <c r="G73" s="32"/>
-      <c r="H73" s="32"/>
-      <c r="I73" s="31"/>
+      <c r="F73" s="37"/>
+      <c r="G73" s="38"/>
+      <c r="H73" s="38"/>
+      <c r="I73" s="37"/>
     </row>
     <row r="74" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="30"/>
+      <c r="A74" s="36"/>
       <c r="B74" s="9">
         <v>6</v>
       </c>
-      <c r="C74" s="31"/>
+      <c r="C74" s="37"/>
       <c r="D74" s="10" t="s">
         <v>131</v>
       </c>
       <c r="E74" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F74" s="31"/>
-      <c r="G74" s="32"/>
-      <c r="H74" s="32"/>
-      <c r="I74" s="31"/>
+      <c r="F74" s="37"/>
+      <c r="G74" s="38"/>
+      <c r="H74" s="38"/>
+      <c r="I74" s="37"/>
     </row>
     <row r="75" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="30"/>
+      <c r="A75" s="36"/>
       <c r="B75" s="7">
         <v>6</v>
       </c>
-      <c r="C75" s="31" t="s">
+      <c r="C75" s="37" t="s">
         <v>132</v>
       </c>
       <c r="D75" s="8" t="s">
@@ -2893,77 +2893,77 @@
       <c r="E75" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F75" s="31" t="s">
+      <c r="F75" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G75" s="32" t="s">
+      <c r="G75" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="H75" s="32" t="str">
+      <c r="H75" s="38" t="str">
         <f>EQUIPO!$B$7</f>
         <v>Jose Espinoza Rivadeneira</v>
       </c>
-      <c r="I75" s="31" t="s">
+      <c r="I75" s="37" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="30"/>
+      <c r="A76" s="36"/>
       <c r="B76" s="9">
         <v>6</v>
       </c>
-      <c r="C76" s="31"/>
+      <c r="C76" s="37"/>
       <c r="D76" s="10" t="s">
         <v>135</v>
       </c>
       <c r="E76" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F76" s="31"/>
-      <c r="G76" s="32"/>
-      <c r="H76" s="32"/>
-      <c r="I76" s="31"/>
+      <c r="F76" s="37"/>
+      <c r="G76" s="38"/>
+      <c r="H76" s="38"/>
+      <c r="I76" s="37"/>
     </row>
     <row r="77" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="30"/>
+      <c r="A77" s="36"/>
       <c r="B77" s="9">
         <v>6</v>
       </c>
-      <c r="C77" s="31"/>
+      <c r="C77" s="37"/>
       <c r="D77" s="10" t="s">
         <v>136</v>
       </c>
       <c r="E77" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F77" s="31"/>
-      <c r="G77" s="32"/>
-      <c r="H77" s="32"/>
-      <c r="I77" s="31"/>
+      <c r="F77" s="37"/>
+      <c r="G77" s="38"/>
+      <c r="H77" s="38"/>
+      <c r="I77" s="37"/>
     </row>
     <row r="78" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A78" s="30"/>
+      <c r="A78" s="36"/>
       <c r="B78" s="9">
         <v>6</v>
       </c>
-      <c r="C78" s="31"/>
+      <c r="C78" s="37"/>
       <c r="D78" s="10" t="s">
         <v>137</v>
       </c>
       <c r="E78" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F78" s="31"/>
-      <c r="G78" s="32"/>
-      <c r="H78" s="32"/>
-      <c r="I78" s="31"/>
+      <c r="F78" s="37"/>
+      <c r="G78" s="38"/>
+      <c r="H78" s="38"/>
+      <c r="I78" s="37"/>
     </row>
     <row r="79" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A79" s="30"/>
+      <c r="A79" s="36"/>
       <c r="B79" s="7">
         <v>6</v>
       </c>
-      <c r="C79" s="31" t="s">
+      <c r="C79" s="37" t="s">
         <v>138</v>
       </c>
       <c r="D79" s="8" t="s">
@@ -2972,73 +2972,73 @@
       <c r="E79" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F79" s="31" t="s">
+      <c r="F79" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G79" s="32" t="s">
+      <c r="G79" s="38" t="s">
         <v>140</v>
       </c>
-      <c r="H79" s="32" t="str">
+      <c r="H79" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I79" s="31" t="s">
+      <c r="I79" s="37" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="30"/>
+      <c r="A80" s="36"/>
       <c r="B80" s="9">
         <v>6</v>
       </c>
-      <c r="C80" s="31"/>
+      <c r="C80" s="37"/>
       <c r="D80" s="10" t="s">
         <v>141</v>
       </c>
       <c r="E80" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F80" s="31"/>
-      <c r="G80" s="32"/>
-      <c r="H80" s="32"/>
-      <c r="I80" s="31"/>
+      <c r="F80" s="37"/>
+      <c r="G80" s="38"/>
+      <c r="H80" s="38"/>
+      <c r="I80" s="37"/>
     </row>
     <row r="81" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A81" s="30"/>
+      <c r="A81" s="36"/>
       <c r="B81" s="9">
         <v>6</v>
       </c>
-      <c r="C81" s="31"/>
+      <c r="C81" s="37"/>
       <c r="D81" s="10" t="s">
         <v>142</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F81" s="31"/>
-      <c r="G81" s="32"/>
-      <c r="H81" s="32"/>
-      <c r="I81" s="31"/>
+      <c r="F81" s="37"/>
+      <c r="G81" s="38"/>
+      <c r="H81" s="38"/>
+      <c r="I81" s="37"/>
     </row>
     <row r="82" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="30"/>
+      <c r="A82" s="36"/>
       <c r="B82" s="9">
         <v>6</v>
       </c>
-      <c r="C82" s="31"/>
+      <c r="C82" s="37"/>
       <c r="D82" s="10" t="s">
         <v>143</v>
       </c>
       <c r="E82" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F82" s="31"/>
-      <c r="G82" s="32"/>
-      <c r="H82" s="32"/>
-      <c r="I82" s="31"/>
+      <c r="F82" s="37"/>
+      <c r="G82" s="38"/>
+      <c r="H82" s="38"/>
+      <c r="I82" s="37"/>
     </row>
     <row r="83" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="33" t="s">
+      <c r="A83" s="32" t="s">
         <v>144</v>
       </c>
       <c r="B83" s="3">
@@ -3068,7 +3068,7 @@
       </c>
     </row>
     <row r="84" spans="1:9" ht="52.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="33"/>
+      <c r="A84" s="32"/>
       <c r="B84" s="5">
         <v>7</v>
       </c>
@@ -3085,7 +3085,7 @@
       <c r="I84" s="34"/>
     </row>
     <row r="85" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A85" s="33"/>
+      <c r="A85" s="32"/>
       <c r="B85" s="5">
         <v>7</v>
       </c>
@@ -3102,7 +3102,7 @@
       <c r="I85" s="34"/>
     </row>
     <row r="86" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A86" s="33"/>
+      <c r="A86" s="32"/>
       <c r="B86" s="5">
         <v>7</v>
       </c>
@@ -3119,7 +3119,7 @@
       <c r="I86" s="34"/>
     </row>
     <row r="87" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A87" s="33"/>
+      <c r="A87" s="32"/>
       <c r="B87" s="3">
         <v>7</v>
       </c>
@@ -3147,7 +3147,7 @@
       </c>
     </row>
     <row r="88" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="33"/>
+      <c r="A88" s="32"/>
       <c r="B88" s="5">
         <v>7</v>
       </c>
@@ -3164,7 +3164,7 @@
       <c r="I88" s="34"/>
     </row>
     <row r="89" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="33"/>
+      <c r="A89" s="32"/>
       <c r="B89" s="5">
         <v>7</v>
       </c>
@@ -3181,7 +3181,7 @@
       <c r="I89" s="34"/>
     </row>
     <row r="90" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="33"/>
+      <c r="A90" s="32"/>
       <c r="B90" s="5">
         <v>7</v>
       </c>
@@ -3198,7 +3198,7 @@
       <c r="I90" s="34"/>
     </row>
     <row r="91" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="33"/>
+      <c r="A91" s="32"/>
       <c r="B91" s="3">
         <v>7</v>
       </c>
@@ -3226,7 +3226,7 @@
       </c>
     </row>
     <row r="92" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A92" s="33"/>
+      <c r="A92" s="32"/>
       <c r="B92" s="5">
         <v>7</v>
       </c>
@@ -3243,7 +3243,7 @@
       <c r="I92" s="34"/>
     </row>
     <row r="93" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A93" s="33"/>
+      <c r="A93" s="32"/>
       <c r="B93" s="5">
         <v>7</v>
       </c>
@@ -3260,7 +3260,7 @@
       <c r="I93" s="34"/>
     </row>
     <row r="94" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A94" s="33"/>
+      <c r="A94" s="32"/>
       <c r="B94" s="5">
         <v>7</v>
       </c>
@@ -3277,13 +3277,13 @@
       <c r="I94" s="34"/>
     </row>
     <row r="95" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A95" s="30" t="s">
+      <c r="A95" s="36" t="s">
         <v>163</v>
       </c>
       <c r="B95" s="7">
         <v>8</v>
       </c>
-      <c r="C95" s="31" t="s">
+      <c r="C95" s="37" t="s">
         <v>164</v>
       </c>
       <c r="D95" s="8" t="s">
@@ -3292,77 +3292,77 @@
       <c r="E95" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F95" s="31" t="s">
+      <c r="F95" s="37" t="s">
         <v>67</v>
       </c>
-      <c r="G95" s="32" t="s">
+      <c r="G95" s="38" t="s">
         <v>166</v>
       </c>
-      <c r="H95" s="32" t="str">
+      <c r="H95" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I95" s="31" t="s">
+      <c r="I95" s="37" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="96" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A96" s="30"/>
+      <c r="A96" s="36"/>
       <c r="B96" s="9">
         <v>8</v>
       </c>
-      <c r="C96" s="31"/>
+      <c r="C96" s="37"/>
       <c r="D96" s="10" t="s">
         <v>167</v>
       </c>
       <c r="E96" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F96" s="31"/>
-      <c r="G96" s="32"/>
-      <c r="H96" s="32"/>
-      <c r="I96" s="31"/>
+      <c r="F96" s="37"/>
+      <c r="G96" s="38"/>
+      <c r="H96" s="38"/>
+      <c r="I96" s="37"/>
     </row>
     <row r="97" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A97" s="30"/>
+      <c r="A97" s="36"/>
       <c r="B97" s="9">
         <v>8</v>
       </c>
-      <c r="C97" s="31"/>
+      <c r="C97" s="37"/>
       <c r="D97" s="10" t="s">
         <v>168</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F97" s="31"/>
-      <c r="G97" s="32"/>
-      <c r="H97" s="32"/>
-      <c r="I97" s="31"/>
+      <c r="F97" s="37"/>
+      <c r="G97" s="38"/>
+      <c r="H97" s="38"/>
+      <c r="I97" s="37"/>
     </row>
     <row r="98" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A98" s="30"/>
+      <c r="A98" s="36"/>
       <c r="B98" s="9">
         <v>8</v>
       </c>
-      <c r="C98" s="31"/>
+      <c r="C98" s="37"/>
       <c r="D98" s="10" t="s">
         <v>169</v>
       </c>
       <c r="E98" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F98" s="31"/>
-      <c r="G98" s="32"/>
-      <c r="H98" s="32"/>
-      <c r="I98" s="31"/>
+      <c r="F98" s="37"/>
+      <c r="G98" s="38"/>
+      <c r="H98" s="38"/>
+      <c r="I98" s="37"/>
     </row>
     <row r="99" spans="1:9" ht="37.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A99" s="30"/>
+      <c r="A99" s="36"/>
       <c r="B99" s="7">
         <v>8</v>
       </c>
-      <c r="C99" s="31" t="s">
+      <c r="C99" s="37" t="s">
         <v>170</v>
       </c>
       <c r="D99" s="8" t="s">
@@ -3371,74 +3371,181 @@
       <c r="E99" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F99" s="31" t="s">
+      <c r="F99" s="37" t="s">
         <v>172</v>
       </c>
-      <c r="G99" s="32" t="s">
+      <c r="G99" s="38" t="s">
         <v>173</v>
       </c>
-      <c r="H99" s="32" t="str">
+      <c r="H99" s="38" t="str">
         <f>EQUIPO!$B$8</f>
         <v>Jack</v>
       </c>
-      <c r="I99" s="31" t="s">
+      <c r="I99" s="37" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="100" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A100" s="30"/>
+      <c r="A100" s="36"/>
       <c r="B100" s="9">
         <v>8</v>
       </c>
-      <c r="C100" s="31"/>
+      <c r="C100" s="37"/>
       <c r="D100" s="10" t="s">
         <v>174</v>
       </c>
       <c r="E100" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F100" s="31"/>
-      <c r="G100" s="32"/>
-      <c r="H100" s="32"/>
-      <c r="I100" s="31"/>
+      <c r="F100" s="37"/>
+      <c r="G100" s="38"/>
+      <c r="H100" s="38"/>
+      <c r="I100" s="37"/>
     </row>
     <row r="101" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A101" s="30"/>
+      <c r="A101" s="36"/>
       <c r="B101" s="9">
         <v>8</v>
       </c>
-      <c r="C101" s="31"/>
+      <c r="C101" s="37"/>
       <c r="D101" s="10" t="s">
         <v>175</v>
       </c>
       <c r="E101" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F101" s="31"/>
-      <c r="G101" s="32"/>
-      <c r="H101" s="32"/>
-      <c r="I101" s="31"/>
+      <c r="F101" s="37"/>
+      <c r="G101" s="38"/>
+      <c r="H101" s="38"/>
+      <c r="I101" s="37"/>
     </row>
     <row r="102" spans="1:9" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A102" s="30"/>
+      <c r="A102" s="36"/>
       <c r="B102" s="9">
         <v>8</v>
       </c>
-      <c r="C102" s="31"/>
+      <c r="C102" s="37"/>
       <c r="D102" s="10" t="s">
         <v>176</v>
       </c>
       <c r="E102" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F102" s="31"/>
-      <c r="G102" s="32"/>
-      <c r="H102" s="32"/>
-      <c r="I102" s="31"/>
+      <c r="F102" s="37"/>
+      <c r="G102" s="38"/>
+      <c r="H102" s="38"/>
+      <c r="I102" s="37"/>
     </row>
   </sheetData>
   <autoFilter ref="A5:I102" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="131">
+    <mergeCell ref="A95:A102"/>
+    <mergeCell ref="C95:C98"/>
+    <mergeCell ref="F95:F98"/>
+    <mergeCell ref="G95:G98"/>
+    <mergeCell ref="H95:H98"/>
+    <mergeCell ref="I95:I98"/>
+    <mergeCell ref="C99:C102"/>
+    <mergeCell ref="F99:F102"/>
+    <mergeCell ref="G99:G102"/>
+    <mergeCell ref="H99:H102"/>
+    <mergeCell ref="I99:I102"/>
+    <mergeCell ref="A83:A94"/>
+    <mergeCell ref="C83:C86"/>
+    <mergeCell ref="F83:F86"/>
+    <mergeCell ref="G83:G86"/>
+    <mergeCell ref="H83:H86"/>
+    <mergeCell ref="I83:I86"/>
+    <mergeCell ref="C87:C90"/>
+    <mergeCell ref="F87:F90"/>
+    <mergeCell ref="G87:G90"/>
+    <mergeCell ref="H87:H90"/>
+    <mergeCell ref="I87:I90"/>
+    <mergeCell ref="C91:C94"/>
+    <mergeCell ref="F91:F94"/>
+    <mergeCell ref="G91:G94"/>
+    <mergeCell ref="H91:H94"/>
+    <mergeCell ref="I91:I94"/>
+    <mergeCell ref="A71:A82"/>
+    <mergeCell ref="C71:C74"/>
+    <mergeCell ref="F71:F74"/>
+    <mergeCell ref="G71:G74"/>
+    <mergeCell ref="H71:H74"/>
+    <mergeCell ref="I71:I74"/>
+    <mergeCell ref="C75:C78"/>
+    <mergeCell ref="F75:F78"/>
+    <mergeCell ref="G75:G78"/>
+    <mergeCell ref="H75:H78"/>
+    <mergeCell ref="I75:I78"/>
+    <mergeCell ref="C79:C82"/>
+    <mergeCell ref="F79:F82"/>
+    <mergeCell ref="G79:G82"/>
+    <mergeCell ref="H79:H82"/>
+    <mergeCell ref="I79:I82"/>
+    <mergeCell ref="A59:A70"/>
+    <mergeCell ref="C59:C62"/>
+    <mergeCell ref="F59:F62"/>
+    <mergeCell ref="G59:G62"/>
+    <mergeCell ref="H59:H62"/>
+    <mergeCell ref="I59:I62"/>
+    <mergeCell ref="C63:C66"/>
+    <mergeCell ref="F63:F66"/>
+    <mergeCell ref="G63:G66"/>
+    <mergeCell ref="H63:H66"/>
+    <mergeCell ref="I63:I66"/>
+    <mergeCell ref="C67:C70"/>
+    <mergeCell ref="F67:F70"/>
+    <mergeCell ref="G67:G70"/>
+    <mergeCell ref="H67:H70"/>
+    <mergeCell ref="I67:I70"/>
+    <mergeCell ref="A47:A58"/>
+    <mergeCell ref="C47:C50"/>
+    <mergeCell ref="F47:F50"/>
+    <mergeCell ref="G47:G50"/>
+    <mergeCell ref="H47:H50"/>
+    <mergeCell ref="I47:I50"/>
+    <mergeCell ref="C51:C54"/>
+    <mergeCell ref="F51:F54"/>
+    <mergeCell ref="G51:G54"/>
+    <mergeCell ref="H51:H54"/>
+    <mergeCell ref="I51:I54"/>
+    <mergeCell ref="C55:C58"/>
+    <mergeCell ref="F55:F58"/>
+    <mergeCell ref="G55:G58"/>
+    <mergeCell ref="H55:H58"/>
+    <mergeCell ref="I55:I58"/>
+    <mergeCell ref="A34:A46"/>
+    <mergeCell ref="C34:C37"/>
+    <mergeCell ref="F34:F37"/>
+    <mergeCell ref="G34:G37"/>
+    <mergeCell ref="H34:H37"/>
+    <mergeCell ref="I34:I37"/>
+    <mergeCell ref="C38:C42"/>
+    <mergeCell ref="F38:F42"/>
+    <mergeCell ref="G38:G42"/>
+    <mergeCell ref="H38:H42"/>
+    <mergeCell ref="I38:I42"/>
+    <mergeCell ref="C43:C46"/>
+    <mergeCell ref="F43:F46"/>
+    <mergeCell ref="G43:G46"/>
+    <mergeCell ref="H43:H46"/>
+    <mergeCell ref="I43:I46"/>
+    <mergeCell ref="C22:C25"/>
+    <mergeCell ref="F22:F25"/>
+    <mergeCell ref="G22:G25"/>
+    <mergeCell ref="H22:H25"/>
+    <mergeCell ref="I22:I25"/>
+    <mergeCell ref="A26:A33"/>
+    <mergeCell ref="C26:C29"/>
+    <mergeCell ref="F26:F29"/>
+    <mergeCell ref="G26:G29"/>
+    <mergeCell ref="H26:H29"/>
+    <mergeCell ref="I26:I29"/>
+    <mergeCell ref="C30:C33"/>
+    <mergeCell ref="F30:F33"/>
+    <mergeCell ref="G30:G33"/>
+    <mergeCell ref="H30:H33"/>
+    <mergeCell ref="I30:I33"/>
     <mergeCell ref="B1:D1"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="B3:D3"/>
@@ -3463,113 +3570,6 @@
     <mergeCell ref="G18:G21"/>
     <mergeCell ref="H18:H21"/>
     <mergeCell ref="I18:I21"/>
-    <mergeCell ref="C22:C25"/>
-    <mergeCell ref="F22:F25"/>
-    <mergeCell ref="G22:G25"/>
-    <mergeCell ref="H22:H25"/>
-    <mergeCell ref="I22:I25"/>
-    <mergeCell ref="A26:A33"/>
-    <mergeCell ref="C26:C29"/>
-    <mergeCell ref="F26:F29"/>
-    <mergeCell ref="G26:G29"/>
-    <mergeCell ref="H26:H29"/>
-    <mergeCell ref="I26:I29"/>
-    <mergeCell ref="C30:C33"/>
-    <mergeCell ref="F30:F33"/>
-    <mergeCell ref="G30:G33"/>
-    <mergeCell ref="H30:H33"/>
-    <mergeCell ref="I30:I33"/>
-    <mergeCell ref="A34:A46"/>
-    <mergeCell ref="C34:C37"/>
-    <mergeCell ref="F34:F37"/>
-    <mergeCell ref="G34:G37"/>
-    <mergeCell ref="H34:H37"/>
-    <mergeCell ref="I34:I37"/>
-    <mergeCell ref="C38:C42"/>
-    <mergeCell ref="F38:F42"/>
-    <mergeCell ref="G38:G42"/>
-    <mergeCell ref="H38:H42"/>
-    <mergeCell ref="I38:I42"/>
-    <mergeCell ref="C43:C46"/>
-    <mergeCell ref="F43:F46"/>
-    <mergeCell ref="G43:G46"/>
-    <mergeCell ref="H43:H46"/>
-    <mergeCell ref="I43:I46"/>
-    <mergeCell ref="A47:A58"/>
-    <mergeCell ref="C47:C50"/>
-    <mergeCell ref="F47:F50"/>
-    <mergeCell ref="G47:G50"/>
-    <mergeCell ref="H47:H50"/>
-    <mergeCell ref="I47:I50"/>
-    <mergeCell ref="C51:C54"/>
-    <mergeCell ref="F51:F54"/>
-    <mergeCell ref="G51:G54"/>
-    <mergeCell ref="H51:H54"/>
-    <mergeCell ref="I51:I54"/>
-    <mergeCell ref="C55:C58"/>
-    <mergeCell ref="F55:F58"/>
-    <mergeCell ref="G55:G58"/>
-    <mergeCell ref="H55:H58"/>
-    <mergeCell ref="I55:I58"/>
-    <mergeCell ref="A59:A70"/>
-    <mergeCell ref="C59:C62"/>
-    <mergeCell ref="F59:F62"/>
-    <mergeCell ref="G59:G62"/>
-    <mergeCell ref="H59:H62"/>
-    <mergeCell ref="I59:I62"/>
-    <mergeCell ref="C63:C66"/>
-    <mergeCell ref="F63:F66"/>
-    <mergeCell ref="G63:G66"/>
-    <mergeCell ref="H63:H66"/>
-    <mergeCell ref="I63:I66"/>
-    <mergeCell ref="C67:C70"/>
-    <mergeCell ref="F67:F70"/>
-    <mergeCell ref="G67:G70"/>
-    <mergeCell ref="H67:H70"/>
-    <mergeCell ref="I67:I70"/>
-    <mergeCell ref="A71:A82"/>
-    <mergeCell ref="C71:C74"/>
-    <mergeCell ref="F71:F74"/>
-    <mergeCell ref="G71:G74"/>
-    <mergeCell ref="H71:H74"/>
-    <mergeCell ref="I71:I74"/>
-    <mergeCell ref="C75:C78"/>
-    <mergeCell ref="F75:F78"/>
-    <mergeCell ref="G75:G78"/>
-    <mergeCell ref="H75:H78"/>
-    <mergeCell ref="I75:I78"/>
-    <mergeCell ref="C79:C82"/>
-    <mergeCell ref="F79:F82"/>
-    <mergeCell ref="G79:G82"/>
-    <mergeCell ref="H79:H82"/>
-    <mergeCell ref="I79:I82"/>
-    <mergeCell ref="A83:A94"/>
-    <mergeCell ref="C83:C86"/>
-    <mergeCell ref="F83:F86"/>
-    <mergeCell ref="G83:G86"/>
-    <mergeCell ref="H83:H86"/>
-    <mergeCell ref="I83:I86"/>
-    <mergeCell ref="C87:C90"/>
-    <mergeCell ref="F87:F90"/>
-    <mergeCell ref="G87:G90"/>
-    <mergeCell ref="H87:H90"/>
-    <mergeCell ref="I87:I90"/>
-    <mergeCell ref="C91:C94"/>
-    <mergeCell ref="F91:F94"/>
-    <mergeCell ref="G91:G94"/>
-    <mergeCell ref="H91:H94"/>
-    <mergeCell ref="I91:I94"/>
-    <mergeCell ref="A95:A102"/>
-    <mergeCell ref="C95:C98"/>
-    <mergeCell ref="F95:F98"/>
-    <mergeCell ref="G95:G98"/>
-    <mergeCell ref="H95:H98"/>
-    <mergeCell ref="I95:I98"/>
-    <mergeCell ref="C99:C102"/>
-    <mergeCell ref="F99:F102"/>
-    <mergeCell ref="G99:G102"/>
-    <mergeCell ref="H99:H102"/>
-    <mergeCell ref="I99:I102"/>
   </mergeCells>
   <conditionalFormatting sqref="E6:E102">
     <cfRule type="expression" dxfId="2" priority="2">
@@ -3625,32 +3625,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>177</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
     </row>
     <row r="2" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="3" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="38" t="s">
+      <c r="A3" s="40" t="s">
         <v>178</v>
       </c>
-      <c r="B3" s="38"/>
-      <c r="C3" s="38"/>
-      <c r="D3" s="38"/>
-      <c r="E3" s="38"/>
-      <c r="F3" s="38"/>
+      <c r="B3" s="40"/>
+      <c r="C3" s="40"/>
+      <c r="D3" s="40"/>
+      <c r="E3" s="40"/>
+      <c r="F3" s="40"/>
     </row>
     <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -3857,29 +3857,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>208</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
     </row>
     <row r="3" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="39" t="s">
+      <c r="A3" s="41" t="s">
         <v>209</v>
       </c>
-      <c r="B3" s="39"/>
-      <c r="C3" s="39"/>
-      <c r="D3" s="39"/>
-      <c r="E3" s="39"/>
+      <c r="B3" s="41"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
     </row>
     <row r="5" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -3942,13 +3942,13 @@
       <c r="E8" s="16"/>
     </row>
     <row r="12" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="40" t="s">
+      <c r="A12" s="42" t="s">
         <v>224</v>
       </c>
-      <c r="B12" s="40"/>
-      <c r="C12" s="40"/>
-      <c r="D12" s="40"/>
-      <c r="E12" s="40"/>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3976,35 +3976,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" s="37" t="s">
+      <c r="A1" s="39" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="37"/>
-      <c r="C1" s="37"/>
-      <c r="D1" s="37"/>
-      <c r="E1" s="37"/>
-      <c r="F1" s="37"/>
-      <c r="G1" s="37"/>
+      <c r="B1" s="39"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="37"/>
-      <c r="B2" s="37"/>
-      <c r="C2" s="37"/>
-      <c r="D2" s="37"/>
-      <c r="E2" s="37"/>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
+      <c r="A2" s="39"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
     </row>
     <row r="3" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="41" t="s">
+      <c r="A3" s="43" t="s">
         <v>226</v>
       </c>
-      <c r="B3" s="41"/>
-      <c r="C3" s="41"/>
-      <c r="D3" s="41"/>
-      <c r="E3" s="41"/>
-      <c r="F3" s="41"/>
-      <c r="G3" s="41"/>
+      <c r="B3" s="43"/>
+      <c r="C3" s="43"/>
+      <c r="D3" s="43"/>
+      <c r="E3" s="43"/>
+      <c r="F3" s="43"/>
+      <c r="G3" s="43"/>
     </row>
     <row r="5" spans="1:7" ht="16.8" x14ac:dyDescent="0.3">
       <c r="A5" s="17" t="s">
@@ -4041,11 +4041,11 @@
       </c>
       <c r="C7" s="20">
         <f>COUNTIFS(PLANIFICACION!$B$6:$B$300,$A7,PLANIFICACION!$E$6:$E$300,"Completado")</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D7" s="20">
         <f>COUNTIFS(PLANIFICACION!$B$6:$B$300,$A7,PLANIFICACION!$E$6:$E$300,"En proceso")</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E7" s="20">
         <f>COUNTIFS(PLANIFICACION!$B$6:$B$300,$A7,PLANIFICACION!$E$6:$E$300,"Falta")</f>
@@ -4053,7 +4053,7 @@
       </c>
       <c r="F7" s="21">
         <f t="shared" ref="F7:F15" si="0">IF(B7=0,0,C7/B7)</f>
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
@@ -4241,11 +4241,11 @@
       </c>
       <c r="C15" s="25">
         <f>SUM(C7:C14)</f>
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="D15" s="25">
         <f>SUM(D7:D14)</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E15" s="25">
         <f>SUM(E7:E14)</f>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="F15" s="26">
         <f t="shared" si="0"/>
-        <v>0.13402061855670103</v>
+        <v>0.16494845360824742</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="16.8" x14ac:dyDescent="0.3">

</xml_diff>